<commit_message>
Removed J2 from position file.
</commit_message>
<xml_diff>
--- a/DC-34-CPEC-Mech-SAO-Rev01p1-CPL_JLCSMT.xlsx
+++ b/DC-34-CPEC-Mech-SAO-Rev01p1-CPL_JLCSMT.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="26">
   <si>
     <t xml:space="preserve">Designator</t>
   </si>
@@ -98,9 +98,6 @@
   </si>
   <si>
     <t xml:space="preserve">D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J2</t>
   </si>
 </sst>
 </file>
@@ -5107,259 +5104,49 @@
       </c>
     </row>
     <row r="287" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A287" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B287" s="0" t="n">
-        <v>126.260056</v>
-      </c>
-      <c r="C287" s="0" t="n">
-        <v>-56.800747</v>
-      </c>
-      <c r="D287" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E287" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D287" s="2"/>
     </row>
     <row r="288" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A288" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B288" s="0" t="n">
-        <v>160.507742</v>
-      </c>
-      <c r="C288" s="0" t="n">
-        <v>-145.660849</v>
-      </c>
-      <c r="D288" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E288" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D288" s="2"/>
     </row>
     <row r="289" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A289" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B289" s="0" t="n">
-        <v>194.755884</v>
-      </c>
-      <c r="C289" s="0" t="n">
-        <v>-101.230981</v>
-      </c>
-      <c r="D289" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E289" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D289" s="2"/>
     </row>
     <row r="290" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A290" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B290" s="0" t="n">
-        <v>126.259752</v>
-      </c>
-      <c r="C290" s="0" t="n">
-        <v>-145.660727</v>
-      </c>
-      <c r="D290" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E290" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D290" s="2"/>
     </row>
     <row r="291" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A291" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B291" s="0" t="n">
-        <v>57.763772</v>
-      </c>
-      <c r="C291" s="0" t="n">
-        <v>-145.660483</v>
-      </c>
-      <c r="D291" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E291" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D291" s="2"/>
     </row>
     <row r="292" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A292" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B292" s="0" t="n">
-        <v>194.755732</v>
-      </c>
-      <c r="C292" s="0" t="n">
-        <v>-145.660971</v>
-      </c>
-      <c r="D292" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E292" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D292" s="2"/>
     </row>
     <row r="293" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A293" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B293" s="0" t="n">
-        <v>194.756036</v>
-      </c>
-      <c r="C293" s="0" t="n">
-        <v>-56.800991</v>
-      </c>
-      <c r="D293" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E293" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D293" s="2"/>
     </row>
     <row r="294" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A294" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B294" s="0" t="n">
-        <v>57.764076</v>
-      </c>
-      <c r="C294" s="0" t="n">
-        <v>-56.800503</v>
-      </c>
-      <c r="D294" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E294" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D294" s="2"/>
     </row>
     <row r="295" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A295" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B295" s="0" t="n">
-        <v>92.012066</v>
-      </c>
-      <c r="C295" s="0" t="n">
-        <v>-56.800625</v>
-      </c>
-      <c r="D295" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E295" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D295" s="2"/>
     </row>
     <row r="296" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A296" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B296" s="0" t="n">
-        <v>92.011914</v>
-      </c>
-      <c r="C296" s="0" t="n">
-        <v>-101.230615</v>
-      </c>
-      <c r="D296" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E296" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D296" s="2"/>
     </row>
     <row r="297" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A297" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B297" s="0" t="n">
-        <v>126.259904</v>
-      </c>
-      <c r="C297" s="0" t="n">
-        <v>-101.230737</v>
-      </c>
-      <c r="D297" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E297" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D297" s="2"/>
     </row>
     <row r="298" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A298" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B298" s="0" t="n">
-        <v>160.507894</v>
-      </c>
-      <c r="C298" s="0" t="n">
-        <v>-101.230859</v>
-      </c>
-      <c r="D298" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E298" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D298" s="2"/>
     </row>
     <row r="299" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A299" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B299" s="0" t="n">
-        <v>160.508046</v>
-      </c>
-      <c r="C299" s="0" t="n">
-        <v>-56.800869</v>
-      </c>
-      <c r="D299" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E299" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D299" s="2"/>
     </row>
     <row r="300" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A300" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B300" s="0" t="n">
-        <v>57.763924</v>
-      </c>
-      <c r="C300" s="0" t="n">
-        <v>-101.230493</v>
-      </c>
-      <c r="D300" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E300" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D300" s="2"/>
     </row>
     <row r="301" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A301" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B301" s="0" t="n">
-        <v>92.011762</v>
-      </c>
-      <c r="C301" s="0" t="n">
-        <v>-145.660605</v>
-      </c>
-      <c r="D301" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E301" s="0" t="n">
-        <v>0</v>
-      </c>
+      <c r="D301" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>